<commit_message>
update matriks dan menambahkan gitignore
</commit_message>
<xml_diff>
--- a/Research Setup/Matriks_Penelitian.xlsx
+++ b/Research Setup/Matriks_Penelitian.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Habbi Widagdo\Documents\Tugas Akhir\Proposal TA\Research Setup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E433EA-D3E3-4205-9F43-55E163E3130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE235F8A-DA5B-4E6C-95AD-C1B289687E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Masalah</t>
   </si>
@@ -39,94 +39,6 @@
     <t>Matriks Penelitian</t>
   </si>
   <si>
-    <t>Terdapat ketidakseimbangan kelas (class imbalance) yang sangat ekstrem  (94% OFF berbanding 6% ON) pada status operasional aktuator nutrients_adder di dataset hidroponik.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Bagaimana penerapan algoritma </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Random Forest</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> dan teknik </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>resampling</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> SMOTE-Tomek dalam mengklasifikasikan status aktuator pada dataset sensor IoT hidroponik yang ekstrem tidak seimbang?</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">2. Bagaimana perbandingan performa model klasifikasi antara data </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>baseline</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> dengan data hasil SMOTE-Tomek berdasarkan metrik evaluasi kelas minoritas?</t>
-    </r>
-  </si>
-  <si>
-    <t>Menerapkan teknik resampling hibrida SMOTE-Tomek (kombinasi oversampling dan pembersihan noise di batas keputusan) pada data latih (training set).</t>
-  </si>
-  <si>
-    <t>Random Forest (algoritma berbasis pohon keputusan/ensemble learning)</t>
-  </si>
-  <si>
-    <t>Precision, Recall, F1-Score, Accuracy (masih di pertimbangkan), dan AUC-PR</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Tujuan</t>
   </si>
   <si>
@@ -142,7 +54,321 @@
     <t>Pemetaan Penelitian yang akan Dilakukan Berdasarkan Matriks Posisi</t>
   </si>
   <si>
-    <t>1.</t>
+    <t>Keseimbangan kelas dapat menghasilkan bias dan mempengaruhi performa model klasifikasi. Model dapat lebih dominan terhadap kelas mayoritas dan gagal mendeteksi informasi penting kelas minoritas.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Untuk mengetahui penerapan teknik penanganan </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>imbalance data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dan </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>machine learning</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pada tugas klasifikasi di domain </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>smart farming</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Untuk mengatahui pengaruh teknik penanganan </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>imbalance data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> terhadap performa model melalui metrik evaluasi.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bagaimana penerapan model machine learning dan teknik penanganan </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>imbalance data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pada domain </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">smart farming </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>untuk tugas klasifikasi?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sejauh mana teknik penanganan </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>imbalance data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> meningkatkan metrik evaluasi </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>machine learning</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>Random Forest</t>
+  </si>
+  <si>
+    <t>SMOTE - Tomek Links</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Hasil evaluasi model yang mendapatkan perlakuan teknik penanganan </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>imbalance data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &gt; Hasil evaluasi model tanpa perlakuan teknik penanganan </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>imbalance data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Hasil penelitian diharapkan dapat membuktikan metode/teknik penanganan </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>imbalance data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pada domaian </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">smart farming </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>dapat diterapkan untuk menghasilkan model dengan performa terbaik</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Precision, Recall, F1-Score, Accuracy (masih di pertimbangkan), MCC, dan AUC-PR</t>
+  </si>
+  <si>
+    <t>Referensi Pendukung</t>
+  </si>
+  <si>
+    <t>Iwan Binanto et al. "The Effect of Data Balancing on Performance of Support Vector Machine and Random Forest Classification for Typhonium Flagelliforme Lodd Dataset"</t>
+  </si>
+  <si>
+    <t>Nitesh V. Chawla et al. "SMOTE: Synthetic Minority Over-sampling Technique"</t>
+  </si>
+  <si>
+    <t>Ivan Tomek. "An Experiment with the Condensed Nearest-Neighbor Rule (Two Modifications of CNN)"</t>
   </si>
 </sst>
 </file>
@@ -214,7 +440,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -222,23 +448,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -520,109 +752,130 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.140625" customWidth="1"/>
-    <col min="2" max="8" width="27.140625" customWidth="1"/>
+    <col min="1" max="8" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:8" s="6" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="1" customFormat="1" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="2" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7"/>
+      <c r="B6" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-    </row>
-    <row r="3" spans="1:8" s="8" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="1" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="7"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
+      <c r="H6" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="2" customFormat="1" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="5" t="s">
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A5:A7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>